<commit_message>
Actualizacao dos graficos e dados
</commit_message>
<xml_diff>
--- a/Lista_Monapo_Turmas.xlsx
+++ b/Lista_Monapo_Turmas.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://muvamozorg.sharepoint.com/sites/mis.drive/Documentos Partilhados/PROJECTOS/Sistema de Monitoria/NEXUS/2026/Dash_Nexus/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="154" documentId="8_{3974BDCB-D2A5-43A1-9815-8A3ABB62B650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B4014C3-A5D3-4163-A33A-5FF2B65ACE41}"/>
+  <xr:revisionPtr revIDLastSave="171" documentId="8_{3974BDCB-D2A5-43A1-9815-8A3ABB62B650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86DF2F43-789D-4086-B4E5-9FFD160390F6}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{56ACAE1C-7A35-401F-B142-1D9154C2B01F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{56ACAE1C-7A35-401F-B142-1D9154C2B01F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$200</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1195" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1201" uniqueCount="223">
   <si>
     <t>Distrito</t>
   </si>
@@ -428,9 +431,6 @@
     <t>ZAINABO PAULITO PAULO</t>
   </si>
   <si>
-    <t>Paulo Alexandre &amp; Tomas Augusto</t>
-  </si>
-  <si>
     <t>TOPELANE</t>
   </si>
   <si>
@@ -705,6 +705,9 @@
   </si>
   <si>
     <t>JASINTO ROMOALDO VICTORINO</t>
+  </si>
+  <si>
+    <t>ISELIA MIGUEL</t>
   </si>
 </sst>
 </file>
@@ -1187,12 +1190,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7025CE97-D830-406F-99E1-8876D639775D}">
-  <dimension ref="A1:G199"/>
+  <dimension ref="A1:G200"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="29" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="28.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1224,7 +1227,7 @@
         <v>7</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>8</v>
@@ -1245,7 +1248,7 @@
         <v>7</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>8</v>
@@ -1266,7 +1269,7 @@
         <v>7</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>8</v>
@@ -1287,7 +1290,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>8</v>
@@ -1308,7 +1311,7 @@
         <v>7</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>8</v>
@@ -1329,7 +1332,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>8</v>
@@ -1350,7 +1353,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>8</v>
@@ -1371,7 +1374,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>8</v>
@@ -1392,7 +1395,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>8</v>
@@ -1413,7 +1416,7 @@
         <v>7</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>8</v>
@@ -1434,7 +1437,7 @@
         <v>7</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>8</v>
@@ -1455,7 +1458,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>8</v>
@@ -1476,7 +1479,7 @@
         <v>7</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>8</v>
@@ -1497,7 +1500,7 @@
         <v>7</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>8</v>
@@ -1518,7 +1521,7 @@
         <v>7</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>8</v>
@@ -1539,7 +1542,7 @@
         <v>7</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>8</v>
@@ -1560,7 +1563,7 @@
         <v>7</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>8</v>
@@ -1581,7 +1584,7 @@
         <v>7</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>8</v>
@@ -1602,7 +1605,7 @@
         <v>7</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>8</v>
@@ -1623,7 +1626,7 @@
         <v>7</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>8</v>
@@ -1644,7 +1647,7 @@
         <v>7</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>8</v>
@@ -1665,7 +1668,7 @@
         <v>7</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>8</v>
@@ -1686,7 +1689,7 @@
         <v>7</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>8</v>
@@ -1707,7 +1710,7 @@
         <v>7</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>8</v>
@@ -1728,7 +1731,7 @@
         <v>7</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>8</v>
@@ -1749,7 +1752,7 @@
         <v>7</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>8</v>
@@ -2001,7 +2004,7 @@
         <v>7</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>42</v>
@@ -2253,7 +2256,7 @@
         <v>7</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C51" s="4" t="s">
         <v>42</v>
@@ -2673,7 +2676,7 @@
         <v>7</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C71" s="4" t="s">
         <v>72</v>
@@ -2715,7 +2718,7 @@
         <v>7</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C73" s="4" t="s">
         <v>72</v>
@@ -3261,7 +3264,7 @@
         <v>7</v>
       </c>
       <c r="B99" s="10" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C99" s="4" t="s">
         <v>101</v>
@@ -3450,7 +3453,7 @@
         <v>7</v>
       </c>
       <c r="B108" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C108" s="4" t="s">
         <v>101</v>
@@ -3600,14 +3603,14 @@
         <v>104</v>
       </c>
       <c r="C115" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D115" s="4"/>
       <c r="E115" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F115" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G115" s="4" t="s">
         <v>39</v>
@@ -3621,14 +3624,14 @@
         <v>105</v>
       </c>
       <c r="C116" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D116" s="4"/>
       <c r="E116" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F116" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G116" s="4" t="s">
         <v>39</v>
@@ -3642,14 +3645,14 @@
         <v>106</v>
       </c>
       <c r="C117" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D117" s="4"/>
       <c r="E117" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F117" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G117" s="4" t="s">
         <v>39</v>
@@ -3663,14 +3666,14 @@
         <v>107</v>
       </c>
       <c r="C118" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D118" s="4"/>
       <c r="E118" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F118" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G118" s="4" t="s">
         <v>39</v>
@@ -3684,14 +3687,14 @@
         <v>108</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D119" s="4"/>
       <c r="E119" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F119" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G119" s="4" t="s">
         <v>39</v>
@@ -3705,14 +3708,14 @@
         <v>109</v>
       </c>
       <c r="C120" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D120" s="4"/>
       <c r="E120" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F120" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G120" s="4" t="s">
         <v>39</v>
@@ -3723,17 +3726,17 @@
         <v>7</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C121" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D121" s="4"/>
       <c r="E121" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F121" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G121" s="4" t="s">
         <v>39</v>
@@ -3747,14 +3750,14 @@
         <v>110</v>
       </c>
       <c r="C122" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D122" s="4"/>
       <c r="E122" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F122" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G122" s="4" t="s">
         <v>39</v>
@@ -3768,14 +3771,14 @@
         <v>111</v>
       </c>
       <c r="C123" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D123" s="4"/>
       <c r="E123" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F123" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G123" s="4" t="s">
         <v>39</v>
@@ -3789,14 +3792,14 @@
         <v>112</v>
       </c>
       <c r="C124" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D124" s="4"/>
       <c r="E124" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F124" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G124" s="4" t="s">
         <v>39</v>
@@ -3810,14 +3813,14 @@
         <v>113</v>
       </c>
       <c r="C125" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D125" s="4"/>
       <c r="E125" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F125" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G125" s="4" t="s">
         <v>39</v>
@@ -3831,14 +3834,14 @@
         <v>114</v>
       </c>
       <c r="C126" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D126" s="4"/>
       <c r="E126" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F126" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G126" s="4" t="s">
         <v>39</v>
@@ -3852,14 +3855,14 @@
         <v>115</v>
       </c>
       <c r="C127" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D127" s="4"/>
       <c r="E127" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F127" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G127" s="4" t="s">
         <v>39</v>
@@ -3873,14 +3876,14 @@
         <v>116</v>
       </c>
       <c r="C128" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D128" s="4"/>
       <c r="E128" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F128" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G128" s="4" t="s">
         <v>39</v>
@@ -3894,14 +3897,14 @@
         <v>117</v>
       </c>
       <c r="C129" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D129" s="4"/>
       <c r="E129" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F129" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G129" s="4" t="s">
         <v>39</v>
@@ -3915,14 +3918,14 @@
         <v>118</v>
       </c>
       <c r="C130" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D130" s="4"/>
       <c r="E130" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F130" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G130" s="4" t="s">
         <v>39</v>
@@ -3936,14 +3939,14 @@
         <v>119</v>
       </c>
       <c r="C131" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D131" s="4"/>
       <c r="E131" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F131" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G131" s="4" t="s">
         <v>39</v>
@@ -3957,14 +3960,14 @@
         <v>120</v>
       </c>
       <c r="C132" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D132" s="4"/>
       <c r="E132" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F132" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G132" s="4" t="s">
         <v>39</v>
@@ -3978,14 +3981,14 @@
         <v>121</v>
       </c>
       <c r="C133" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D133" s="4"/>
       <c r="E133" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F133" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G133" s="4" t="s">
         <v>39</v>
@@ -3999,14 +4002,14 @@
         <v>122</v>
       </c>
       <c r="C134" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D134" s="4"/>
       <c r="E134" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F134" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G134" s="4" t="s">
         <v>39</v>
@@ -4020,14 +4023,14 @@
         <v>123</v>
       </c>
       <c r="C135" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D135" s="4"/>
       <c r="E135" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F135" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G135" s="4" t="s">
         <v>39</v>
@@ -4041,14 +4044,14 @@
         <v>124</v>
       </c>
       <c r="C136" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D136" s="4"/>
       <c r="E136" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F136" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G136" s="4" t="s">
         <v>39</v>
@@ -4062,14 +4065,14 @@
         <v>125</v>
       </c>
       <c r="C137" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D137" s="4"/>
       <c r="E137" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F137" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G137" s="4" t="s">
         <v>39</v>
@@ -4083,14 +4086,14 @@
         <v>126</v>
       </c>
       <c r="C138" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D138" s="4"/>
       <c r="E138" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F138" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G138" s="4" t="s">
         <v>39</v>
@@ -4104,14 +4107,14 @@
         <v>127</v>
       </c>
       <c r="C139" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D139" s="4"/>
       <c r="E139" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F139" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G139" s="4" t="s">
         <v>39</v>
@@ -4125,14 +4128,14 @@
         <v>128</v>
       </c>
       <c r="C140" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D140" s="4"/>
       <c r="E140" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F140" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G140" s="4" t="s">
         <v>39</v>
@@ -4146,14 +4149,14 @@
         <v>129</v>
       </c>
       <c r="C141" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D141" s="4"/>
       <c r="E141" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F141" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G141" s="4" t="s">
         <v>39</v>
@@ -4164,17 +4167,17 @@
         <v>7</v>
       </c>
       <c r="B142" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C142" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D142" s="4"/>
       <c r="E142" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F142" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G142" s="4" t="s">
         <v>39</v>
@@ -4185,17 +4188,17 @@
         <v>7</v>
       </c>
       <c r="B143" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C143" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D143" s="4"/>
       <c r="E143" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F143" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G143" s="4" t="s">
         <v>39</v>
@@ -4206,10 +4209,10 @@
         <v>7</v>
       </c>
       <c r="B144" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C144" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D144" s="4"/>
       <c r="E144" s="4" t="s">
@@ -4227,10 +4230,10 @@
         <v>7</v>
       </c>
       <c r="B145" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C145" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D145" s="4"/>
       <c r="E145" s="4" t="s">
@@ -4248,10 +4251,10 @@
         <v>7</v>
       </c>
       <c r="B146" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C146" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D146" s="4"/>
       <c r="E146" s="4" t="s">
@@ -4269,10 +4272,10 @@
         <v>7</v>
       </c>
       <c r="B147" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C147" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D147" s="4"/>
       <c r="E147" s="4" t="s">
@@ -4290,10 +4293,10 @@
         <v>7</v>
       </c>
       <c r="B148" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C148" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D148" s="4"/>
       <c r="E148" s="4" t="s">
@@ -4311,10 +4314,10 @@
         <v>7</v>
       </c>
       <c r="B149" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C149" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D149" s="4"/>
       <c r="E149" s="4" t="s">
@@ -4332,10 +4335,10 @@
         <v>7</v>
       </c>
       <c r="B150" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C150" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D150" s="4"/>
       <c r="E150" s="4" t="s">
@@ -4353,10 +4356,10 @@
         <v>7</v>
       </c>
       <c r="B151" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C151" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D151" s="4"/>
       <c r="E151" s="4" t="s">
@@ -4374,10 +4377,10 @@
         <v>7</v>
       </c>
       <c r="B152" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C152" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D152" s="4"/>
       <c r="E152" s="4" t="s">
@@ -4395,10 +4398,10 @@
         <v>7</v>
       </c>
       <c r="B153" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C153" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D153" s="4"/>
       <c r="E153" s="4" t="s">
@@ -4416,10 +4419,10 @@
         <v>7</v>
       </c>
       <c r="B154" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C154" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D154" s="4"/>
       <c r="E154" s="4" t="s">
@@ -4437,10 +4440,10 @@
         <v>7</v>
       </c>
       <c r="B155" s="3" t="s">
-        <v>147</v>
+        <v>222</v>
       </c>
       <c r="C155" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D155" s="4"/>
       <c r="E155" s="4" t="s">
@@ -4458,10 +4461,10 @@
         <v>7</v>
       </c>
       <c r="B156" s="3" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="C156" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D156" s="4"/>
       <c r="E156" s="4" t="s">
@@ -4479,10 +4482,10 @@
         <v>7</v>
       </c>
       <c r="B157" s="3" t="s">
-        <v>159</v>
+        <v>140</v>
       </c>
       <c r="C157" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D157" s="4"/>
       <c r="E157" s="4" t="s">
@@ -4500,10 +4503,10 @@
         <v>7</v>
       </c>
       <c r="B158" s="3" t="s">
-        <v>145</v>
+        <v>158</v>
       </c>
       <c r="C158" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D158" s="4"/>
       <c r="E158" s="4" t="s">
@@ -4521,10 +4524,10 @@
         <v>7</v>
       </c>
       <c r="B159" s="3" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="C159" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D159" s="4"/>
       <c r="E159" s="4" t="s">
@@ -4542,10 +4545,10 @@
         <v>7</v>
       </c>
       <c r="B160" s="3" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="C160" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D160" s="4"/>
       <c r="E160" s="4" t="s">
@@ -4558,15 +4561,15 @@
         <v>40</v>
       </c>
     </row>
-    <row r="161" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A161" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B161" s="3" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C161" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D161" s="4"/>
       <c r="E161" s="4" t="s">
@@ -4579,15 +4582,15 @@
         <v>40</v>
       </c>
     </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A162" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B162" s="3" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="C162" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D162" s="4"/>
       <c r="E162" s="4" t="s">
@@ -4605,10 +4608,10 @@
         <v>7</v>
       </c>
       <c r="B163" s="3" t="s">
-        <v>134</v>
+        <v>152</v>
       </c>
       <c r="C163" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D163" s="4"/>
       <c r="E163" s="4" t="s">
@@ -4626,10 +4629,10 @@
         <v>7</v>
       </c>
       <c r="B164" s="3" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C164" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D164" s="4"/>
       <c r="E164" s="4" t="s">
@@ -4647,10 +4650,10 @@
         <v>7</v>
       </c>
       <c r="B165" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C165" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D165" s="4"/>
       <c r="E165" s="4" t="s">
@@ -4668,10 +4671,10 @@
         <v>7</v>
       </c>
       <c r="B166" s="3" t="s">
-        <v>158</v>
+        <v>134</v>
       </c>
       <c r="C166" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D166" s="4"/>
       <c r="E166" s="4" t="s">
@@ -4689,10 +4692,10 @@
         <v>7</v>
       </c>
       <c r="B167" s="3" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="C167" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D167" s="4"/>
       <c r="E167" s="4" t="s">
@@ -4710,10 +4713,10 @@
         <v>7</v>
       </c>
       <c r="B168" s="3" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="C168" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D168" s="4"/>
       <c r="E168" s="4" t="s">
@@ -4731,10 +4734,10 @@
         <v>7</v>
       </c>
       <c r="B169" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C169" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D169" s="4"/>
       <c r="E169" s="4" t="s">
@@ -4752,10 +4755,10 @@
         <v>7</v>
       </c>
       <c r="B170" s="3" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C170" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D170" s="4"/>
       <c r="E170" s="4" t="s">
@@ -4768,15 +4771,15 @@
         <v>40</v>
       </c>
     </row>
-    <row r="171" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A171" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B171" s="3" t="s">
-        <v>186</v>
+        <v>139</v>
       </c>
       <c r="C171" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D171" s="4"/>
       <c r="E171" s="4" t="s">
@@ -4789,15 +4792,15 @@
         <v>40</v>
       </c>
     </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A172" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B172" s="3" t="s">
-        <v>166</v>
+        <v>185</v>
       </c>
       <c r="C172" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D172" s="4"/>
       <c r="E172" s="4" t="s">
@@ -4815,20 +4818,20 @@
         <v>7</v>
       </c>
       <c r="B173" s="3" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C173" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D173" s="4"/>
       <c r="E173" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F173" s="4" t="s">
-        <v>130</v>
+        <v>35</v>
       </c>
       <c r="G173" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="174" spans="1:7" x14ac:dyDescent="0.3">
@@ -4839,56 +4842,56 @@
         <v>162</v>
       </c>
       <c r="C174" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D174" s="4"/>
       <c r="E174" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F174" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G174" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="175" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A175" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B175" s="3" t="s">
-        <v>178</v>
+        <v>161</v>
       </c>
       <c r="C175" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D175" s="4"/>
       <c r="E175" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F175" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G175" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A176" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B176" s="3" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="C176" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D176" s="4"/>
       <c r="E176" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F176" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G176" s="4" t="s">
         <v>41</v>
@@ -4899,17 +4902,17 @@
         <v>7</v>
       </c>
       <c r="B177" s="3" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="C177" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D177" s="4"/>
       <c r="E177" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F177" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G177" s="4" t="s">
         <v>41</v>
@@ -4920,17 +4923,17 @@
         <v>7</v>
       </c>
       <c r="B178" s="3" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="C178" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D178" s="4"/>
       <c r="E178" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F178" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G178" s="4" t="s">
         <v>41</v>
@@ -4941,59 +4944,59 @@
         <v>7</v>
       </c>
       <c r="B179" s="3" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="C179" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D179" s="4"/>
       <c r="E179" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F179" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G179" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="180" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A180" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B180" s="3" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="C180" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D180" s="4"/>
       <c r="E180" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F180" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G180" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="181" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A181" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B181" s="3" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C181" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D181" s="4"/>
       <c r="E181" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F181" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G181" s="4" t="s">
         <v>41</v>
@@ -5004,17 +5007,17 @@
         <v>7</v>
       </c>
       <c r="B182" s="3" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="C182" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D182" s="4"/>
       <c r="E182" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F182" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G182" s="4" t="s">
         <v>41</v>
@@ -5025,101 +5028,101 @@
         <v>7</v>
       </c>
       <c r="B183" s="3" t="s">
-        <v>171</v>
+        <v>187</v>
       </c>
       <c r="C183" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D183" s="4"/>
       <c r="E183" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F183" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G183" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="184" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A184" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B184" s="3" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="C184" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D184" s="4"/>
       <c r="E184" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F184" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G184" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A185" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B185" s="3" t="s">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="C185" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D185" s="4"/>
       <c r="E185" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F185" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G185" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="186" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A186" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B186" s="3" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="C186" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D186" s="4"/>
       <c r="E186" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F186" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G186" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A187" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B187" s="3" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="C187" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D187" s="4"/>
       <c r="E187" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F187" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G187" s="4" t="s">
         <v>41</v>
@@ -5130,17 +5133,17 @@
         <v>7</v>
       </c>
       <c r="B188" s="3" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="C188" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D188" s="4"/>
       <c r="E188" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F188" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G188" s="4" t="s">
         <v>41</v>
@@ -5151,17 +5154,17 @@
         <v>7</v>
       </c>
       <c r="B189" s="3" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="C189" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D189" s="4"/>
       <c r="E189" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F189" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G189" s="4" t="s">
         <v>41</v>
@@ -5172,17 +5175,17 @@
         <v>7</v>
       </c>
       <c r="B190" s="3" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="C190" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D190" s="4"/>
       <c r="E190" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F190" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G190" s="4" t="s">
         <v>41</v>
@@ -5193,17 +5196,17 @@
         <v>7</v>
       </c>
       <c r="B191" s="3" t="s">
-        <v>183</v>
+        <v>164</v>
       </c>
       <c r="C191" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D191" s="4"/>
       <c r="E191" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F191" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G191" s="4" t="s">
         <v>41</v>
@@ -5214,17 +5217,17 @@
         <v>7</v>
       </c>
       <c r="B192" s="3" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="C192" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D192" s="4"/>
       <c r="E192" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F192" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G192" s="4" t="s">
         <v>41</v>
@@ -5235,17 +5238,17 @@
         <v>7</v>
       </c>
       <c r="B193" s="3" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="C193" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D193" s="4"/>
       <c r="E193" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F193" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G193" s="4" t="s">
         <v>41</v>
@@ -5256,17 +5259,17 @@
         <v>7</v>
       </c>
       <c r="B194" s="3" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C194" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D194" s="4"/>
       <c r="E194" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F194" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G194" s="4" t="s">
         <v>41</v>
@@ -5277,17 +5280,17 @@
         <v>7</v>
       </c>
       <c r="B195" s="3" t="s">
-        <v>170</v>
+        <v>188</v>
       </c>
       <c r="C195" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D195" s="4"/>
       <c r="E195" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F195" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G195" s="4" t="s">
         <v>41</v>
@@ -5298,17 +5301,17 @@
         <v>7</v>
       </c>
       <c r="B196" s="3" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C196" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D196" s="4"/>
       <c r="E196" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F196" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G196" s="4" t="s">
         <v>41</v>
@@ -5319,17 +5322,17 @@
         <v>7</v>
       </c>
       <c r="B197" s="3" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="C197" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D197" s="4"/>
       <c r="E197" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F197" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G197" s="4" t="s">
         <v>41</v>
@@ -5340,17 +5343,17 @@
         <v>7</v>
       </c>
       <c r="B198" s="3" t="s">
-        <v>177</v>
+        <v>163</v>
       </c>
       <c r="C198" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D198" s="4"/>
       <c r="E198" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F198" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G198" s="4" t="s">
         <v>41</v>
@@ -5361,52 +5364,55 @@
         <v>7</v>
       </c>
       <c r="B199" s="3" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="C199" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D199" s="4"/>
       <c r="E199" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F199" s="4" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="G199" s="4" t="s">
         <v>41</v>
       </c>
     </row>
+    <row r="200" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A200" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B200" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="C200" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="D200" s="4"/>
+      <c r="E200" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F200" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G200" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G199">
-    <sortCondition ref="G1:G199"/>
+  <autoFilter ref="A1:G200" xr:uid="{7025CE97-D830-406F-99E1-8876D639775D}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G200">
+    <sortCondition ref="G1:G200"/>
   </sortState>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100DC8BB5B596CFDD4794B3344F0E8F53A4" ma:contentTypeVersion="15" ma:contentTypeDescription="Criar um novo documento." ma:contentTypeScope="" ma:versionID="9a7078cd21229583650f2264465a1c40">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="20d57abc-823c-4051-a81a-1a0a01a8f39e" xmlns:ns3="54c5ab46-7543-4aba-b0fa-79d6a199bef5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4e45437c47114f519c494620e3e4bb67" ns2:_="" ns3:_="">
     <xsd:import namespace="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
@@ -5641,26 +5647,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA8DEF73-C45F-4508-B6B7-3C4F7ADA892C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
-    <ds:schemaRef ds:uri="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6D7EAF1-4CA4-4623-B746-2AEA826AD603}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5989225A-9688-48E6-A2F1-F1F3D82C6276}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5677,4 +5684,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA8DEF73-C45F-4508-B6B7-3C4F7ADA892C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
+    <ds:schemaRef ds:uri="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6D7EAF1-4CA4-4623-B746-2AEA826AD603}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>